<commit_message>
changed catalog to updated version, including more
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet state="visible" name="catalog" sheetId="1" r:id="rId5"/>
     <sheet state="visible" name="presets" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="raw_imports" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -12,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="68">
   <si>
     <t>id</t>
   </si>
@@ -68,6 +69,9 @@
     <t>sugammadex 200mg 2mL</t>
   </si>
   <si>
+    <t>anexate 0.5mg 5mL</t>
+  </si>
+  <si>
     <t>analgesie</t>
   </si>
   <si>
@@ -98,6 +102,15 @@
     <t>litican 50mg</t>
   </si>
   <si>
+    <t>anti-hypertensiva</t>
+  </si>
+  <si>
+    <t>Rydene 5mg 5mL</t>
+  </si>
+  <si>
+    <t>seloken 5mg 5mL</t>
+  </si>
+  <si>
     <t>noodmedicatie</t>
   </si>
   <si>
@@ -110,6 +123,9 @@
     <t>atropine 1mg 5mL</t>
   </si>
   <si>
+    <t>adrenaline 1mg 10mL</t>
+  </si>
+  <si>
     <t>antibiotica</t>
   </si>
   <si>
@@ -119,6 +135,12 @@
     <t>Amoxiclav 1g</t>
   </si>
   <si>
+    <t>Amoxiclav 500mg</t>
+  </si>
+  <si>
+    <t>Dalacin 600mg</t>
+  </si>
+  <si>
     <t>locale_anesthetica</t>
   </si>
   <si>
@@ -137,10 +159,64 @@
     <t>catapressan 150mcg 2mL</t>
   </si>
   <si>
+    <t>lasix 20mg 2mL</t>
+  </si>
+  <si>
+    <t>magnesiumsulfaat 1g 10mL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">miniplasco 10mL NaCl 0.9% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">miniplasco 20mL NaCl 0.9% </t>
+  </si>
+  <si>
     <t>infuusvloeistof</t>
   </si>
   <si>
     <t>Hartmann 1L</t>
+  </si>
+  <si>
+    <t>$2037--2000030107</t>
+  </si>
+  <si>
+    <t>aerochamber</t>
+  </si>
+  <si>
+    <t>$2037--2005000154</t>
+  </si>
+  <si>
+    <t>amoxicmlav 500mg</t>
+  </si>
+  <si>
+    <t>$2037--2000081167</t>
+  </si>
+  <si>
+    <t>$2037--2000090572</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dalacin C 600mg </t>
+  </si>
+  <si>
+    <t>$2037--2000618018</t>
+  </si>
+  <si>
+    <t>$2037--2001862003</t>
+  </si>
+  <si>
+    <t>$2037--2002017805</t>
+  </si>
+  <si>
+    <t>$2037--2004753993</t>
+  </si>
+  <si>
+    <t>$2037--2004754017</t>
+  </si>
+  <si>
+    <t>$2037--2002229566</t>
+  </si>
+  <si>
+    <t>$2037--2003020824</t>
   </si>
 </sst>
 </file>
@@ -208,6 +284,10 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -416,8 +496,11 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="15.0"/>
-    <col customWidth="1" min="2" max="3" width="25.88"/>
+    <col customWidth="1" min="1" max="1" width="9.38"/>
+    <col customWidth="1" min="2" max="2" width="20.5"/>
+    <col customWidth="1" min="3" max="3" width="25.5"/>
+    <col customWidth="1" min="5" max="5" width="8.75"/>
+    <col customWidth="1" min="7" max="7" width="16.88"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -607,14 +690,14 @@
       <c r="A10" s="2">
         <v>9.0</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="2">
-        <v>2.002505981E9</v>
+      <c r="D10" s="1">
+        <v>2.000090572E9</v>
       </c>
       <c r="F10" s="1">
         <v>1.0</v>
@@ -622,19 +705,21 @@
       <c r="G10" s="3">
         <v>46105.0</v>
       </c>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
     </row>
     <row r="11">
       <c r="A11" s="2">
         <v>10.0</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="B11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>20</v>
       </c>
       <c r="D11" s="2">
-        <v>2.003555027E9</v>
+        <v>2.002505981E9</v>
       </c>
       <c r="F11" s="1">
         <v>1.0</v>
@@ -648,16 +733,16 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>21</v>
       </c>
       <c r="D12" s="2">
-        <v>2.000670621E9</v>
+        <v>2.003555027E9</v>
       </c>
       <c r="F12" s="1">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="G12" s="3">
         <v>46105.0</v>
@@ -668,16 +753,16 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D13" s="2">
-        <v>2.003252153E9</v>
+        <v>2.000670621E9</v>
       </c>
       <c r="F13" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="G13" s="3">
         <v>46105.0</v>
@@ -688,13 +773,13 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="D14" s="2">
-        <v>2.002364314E9</v>
+        <v>2.003252153E9</v>
       </c>
       <c r="F14" s="1">
         <v>1.0</v>
@@ -708,13 +793,13 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D15" s="2">
-        <v>2.000003005E9</v>
+        <v>2.002364314E9</v>
       </c>
       <c r="F15" s="1">
         <v>1.0</v>
@@ -728,13 +813,13 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D16" s="2">
-        <v>2.000634064E9</v>
+        <v>2.000003005E9</v>
       </c>
       <c r="F16" s="1">
         <v>1.0</v>
@@ -748,13 +833,13 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D17" s="2">
-        <v>2.00189295E9</v>
+        <v>2.000634064E9</v>
       </c>
       <c r="F17" s="1">
         <v>1.0</v>
@@ -767,14 +852,14 @@
       <c r="A18" s="2">
         <v>17.0</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="D18" s="2">
-        <v>2.000851759E9</v>
+        <v>2.00189295E9</v>
       </c>
       <c r="F18" s="1">
         <v>1.0</v>
@@ -787,14 +872,14 @@
       <c r="A19" s="2">
         <v>18.0</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>28</v>
+      <c r="B19" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="2">
-        <v>2.002547272E9</v>
+      <c r="D19" s="1">
+        <v>2.002229566E9</v>
       </c>
       <c r="F19" s="1">
         <v>1.0</v>
@@ -807,14 +892,14 @@
       <c r="A20" s="2">
         <v>19.0</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>28</v>
+      <c r="B20" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="2">
-        <v>2.000120973E9</v>
+      <c r="D20" s="1">
+        <v>2.003020824E9</v>
       </c>
       <c r="F20" s="1">
         <v>1.0</v>
@@ -827,14 +912,14 @@
       <c r="A21" s="2">
         <v>20.0</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D21" s="2">
-        <v>2.000439092E9</v>
+        <v>2.000851759E9</v>
       </c>
       <c r="F21" s="1">
         <v>1.0</v>
@@ -847,14 +932,14 @@
       <c r="A22" s="2">
         <v>21.0</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="1" t="s">
         <v>34</v>
       </c>
       <c r="D22" s="2">
-        <v>2.000080961E9</v>
+        <v>2.002547272E9</v>
       </c>
       <c r="F22" s="1">
         <v>1.0</v>
@@ -867,14 +952,14 @@
       <c r="A23" s="2">
         <v>22.0</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="D23" s="2">
-        <v>2.001887513E9</v>
+        <v>2.000120973E9</v>
       </c>
       <c r="F23" s="1">
         <v>1.0</v>
@@ -887,14 +972,14 @@
       <c r="A24" s="2">
         <v>23.0</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>37</v>
+      <c r="B24" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="D24" s="1">
-        <v>2.001887505E9</v>
+        <v>2.000030107E9</v>
       </c>
       <c r="F24" s="1">
         <v>1.0</v>
@@ -908,13 +993,13 @@
         <v>24.0</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="1">
-        <v>2.002887702E9</v>
+      <c r="D25" s="2">
+        <v>2.000439092E9</v>
       </c>
       <c r="F25" s="1">
         <v>1.0</v>
@@ -927,14 +1012,14 @@
       <c r="A26" s="2">
         <v>25.0</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D26" s="1">
-        <v>2.000431008E9</v>
+      <c r="D26" s="2">
+        <v>2.000080961E9</v>
       </c>
       <c r="F26" s="1">
         <v>1.0</v>
@@ -947,21 +1032,225 @@
       <c r="A27" s="2">
         <v>26.0</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="1">
+        <v>2.000081167E9</v>
+      </c>
+      <c r="F27" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G27" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="D28" s="1">
+        <v>2.000618018E9</v>
+      </c>
+      <c r="F28" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G28" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D27" s="1">
+      <c r="C29" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="2">
+        <v>2.001887513E9</v>
+      </c>
+      <c r="F29" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G29" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D30" s="1">
+        <v>2.001887505E9</v>
+      </c>
+      <c r="F30" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G30" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" s="1">
+        <v>2.002887702E9</v>
+      </c>
+      <c r="F31" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G31" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D32" s="1">
+        <v>2.000431008E9</v>
+      </c>
+      <c r="F32" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G32" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D33" s="1">
+        <v>2.001862003E9</v>
+      </c>
+      <c r="F33" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G33" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D34" s="1">
+        <v>2.002017805E9</v>
+      </c>
+      <c r="F34" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G34" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D35" s="1">
+        <v>2.004753993E9</v>
+      </c>
+      <c r="F35" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G35" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D36" s="1">
+        <v>2.004754017E9</v>
+      </c>
+      <c r="F36" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G36" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="1">
         <v>2.004807591E9</v>
       </c>
-      <c r="F27" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="G27" s="3">
-        <v>46105.0</v>
-      </c>
+      <c r="F37" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G37" s="3">
+        <v>46105.0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2"/>
+      <c r="G38" s="3"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -977,4 +1266,104 @@
   <sheetData/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>